<commit_message>
Update soccer trades 2026-07-27 23:01:23 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Europa League_UEFA/trades.xlsx
+++ b/data/sxbet/ligas/Europa League_UEFA/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,23 +531,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xcfc2858bc694fbf8557c05f8f7fd20f59fd4990088d7f08f96947050324a2e61</t>
+          <t>0x9eb4b01eefa201544b1ccdb4c5c6604e0714ac629344d4d2b7b17cc1464fb5c7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFbF8d0BCccedDdAc69C0DC38823fE24842afa03C</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>4.881</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.5337</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -563,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>FC Midtjylland vs Besiktas</t>
+          <t>FC Hradec Kralove vs Tromso</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>FC Hradec Kralove</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>Tromso</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xda06ff264d51913dfda755a8c4a477b88663ff22d289eb6f556018e55bf68d04</t>
+          <t>0xc43fb7b2993be2553cb93dc8bab291577c90b4aa7ac359f3b83149bfa631bb40</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19577560</t>
+          <t>L19577176</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785157337</t>
+          <t>1785189317</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>9.144731</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,27 +635,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x6d9c715f878347d23b5132d44c3d76e250960d8a888670fe9b446ebcef8c5cef</t>
+          <t>0x72247e16c302aa1a252495938a15e1d60e4b267830f4978c0b1e53c944fe7833</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x44cE278A4b373d2bFD26e6a2F5fA4E3550151d67</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFbF8d0BCccedDdAc69C0DC38823fE24842afa03C</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>4.881</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.5337</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -663,11 +659,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Besiktas</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -675,27 +667,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>FC Midtjylland vs Besiktas</t>
+          <t>FC Hradec Kralove vs Tromso</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>FC Hradec Kralove</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>Tromso</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xd45cdb893a2b175b1fae5101e51318244d81038ac8cdd664f9d6b1c4b589d532</t>
+          <t>0xc43fb7b2993be2553cb93dc8bab291577c90b4aa7ac359f3b83149bfa631bb40</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19577560</t>
+          <t>L19577176</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785154148</t>
+          <t>1785188885</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>5.041667</t>
+          <t>9.144731</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,12 +739,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xc10cd30f1ad9ff73882f16291a9858024418214eb562a5dbbad80c0ecae1c52f</t>
+          <t>0x605d65f217cfad8dba3fc5fc8ba81f33c522bb6d2702ab1896e28f2a043e7284</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -762,12 +754,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.36789</t>
+          <t>20.5</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -777,7 +769,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>FC Twente</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -787,27 +779,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>FC Midtjylland vs Besiktas</t>
+          <t>Ferencvaros vs FC Twente</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>FC Twente</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xd45cdb893a2b175b1fae5101e51318244d81038ac8cdd664f9d6b1c4b589d532</t>
+          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19577560</t>
+          <t>L19578664</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +824,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785153790</t>
+          <t>1785186773</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785430800</t>
+          <t>1785436200</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>9.866208</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,12 +851,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x72c1b3c5fcfde9fcf9031572e4700cad5504a7350908921543fd656f10cf9747</t>
+          <t>0x31389f85488fa9e54013f64ac333a2b550d2412b8db664b843e4ce83e7ac4987</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x44cE278A4b373d2bFD26e6a2F5fA4E3550151d67</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -874,12 +866,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>20.5</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -889,7 +881,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>FC Twente</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -899,27 +891,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>FC Midtjylland vs Besiktas</t>
+          <t>Ferencvaros vs FC Twente</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>FC Twente</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xd45cdb893a2b175b1fae5101e51318244d81038ac8cdd664f9d6b1c4b589d532</t>
+          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19577560</t>
+          <t>L19578664</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +936,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785153790</t>
+          <t>1785186621</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1785430800</t>
+          <t>1785436200</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>5.041667</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,12 +963,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xfe31a156d44f9e3b282c8377721b24b01c0625a47209ef8f421fc350af3dac0f</t>
+          <t>0xfb23cf678aafc207af69fb8dfa1e83d0a06b41177f42b72e0eb9221a27e820ba</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x12e3C74BC44f9C2C1f9215a84C3862510219Dd10</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -986,22 +978,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>65.95</t>
+          <t>20.5</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.3713</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Europa League</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove</t>
+          <t>FC Twente</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1011,27 +1003,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove vs Tromso</t>
+          <t>Ferencvaros vs FC Twente</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Tromso</t>
+          <t>FC Twente</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x0d9f7cd21696b245b975157ec565ba91ba0db43a168fd64ff0caebbbec205950</t>
+          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19577176</t>
+          <t>L19578664</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1056,17 +1048,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785131538</t>
+          <t>1785186464</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1785430800</t>
+          <t>1785436200</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>177.643098</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,110 +1075,1102 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>0x3138a3ad46ea4c79099bef4064759debf254c0f7929452594d354137a19e0673</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.41</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Ferencvaros vs FC Twente</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Ferencvaros</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>L19578664</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1785186313</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1785436200</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>0x2f2706b1ff85c18b198514da422a74b19942ac8b11089fe8ede6b98b57fcd6fd</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.41</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Ferencvaros vs FC Twente</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Ferencvaros</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19578664</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1785185868</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1785436200</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0x75d4a8cc9d03da588fcd6106f912b7eb69342da973970aa5144a52fd652df720</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0x8b3809dd81A411A1CcC110e23281D3861E41D439</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.2662</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Ferencvaros vs FC Twente</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Ferencvaros</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0x31485d66881ea25fc18ee05567734ae7ae66fb87f6fcca8575303fab366000be</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>L19578664</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1785182082</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1785436200</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>101.408451</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0xd994586c2c89af6ad574d50a0f8c8700e90e7f22d20bf49a633feaa989af50bf</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>98.9699</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.9187</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Europa League</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>SL Benfica FC</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>SL Benfica FC vs FC St. Gallen</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>SL Benfica FC</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>FC St. Gallen</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0xf1cfaffefafaf6e63eaa25f347bda991a38fb6aa57e14fa84b386fed55a3f99b</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>L19577588</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1785178276</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1785438000</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>107.72234</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0xcfc2858bc694fbf8557c05f8f7fd20f59fd4990088d7f08f96947050324a2e61</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>24.5</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.49</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>FC Midtjylland vs Besiktas</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>FC Midtjylland</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0xda06ff264d51913dfda755a8c4a477b88663ff22d289eb6f556018e55bf68d04</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>L19577560</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1785157337</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1785430800</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>0x6d9c715f878347d23b5132d44c3d76e250960d8a888670fe9b446ebcef8c5cef</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0x44cE278A4b373d2bFD26e6a2F5fA4E3550151d67</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>FC Midtjylland vs Besiktas</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>FC Midtjylland</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0xd45cdb893a2b175b1fae5101e51318244d81038ac8cdd664f9d6b1c4b589d532</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>L19577560</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1785154148</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1785430800</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>5.041667</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>0xc10cd30f1ad9ff73882f16291a9858024418214eb562a5dbbad80c0ecae1c52f</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2.36789</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>FC Midtjylland vs Besiktas</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>FC Midtjylland</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0xd45cdb893a2b175b1fae5101e51318244d81038ac8cdd664f9d6b1c4b589d532</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>L19577560</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1785153790</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>1785430800</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>9.866208</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>0x72c1b3c5fcfde9fcf9031572e4700cad5504a7350908921543fd656f10cf9747</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0x44cE278A4b373d2bFD26e6a2F5fA4E3550151d67</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>FC Midtjylland vs Besiktas</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>FC Midtjylland</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0xd45cdb893a2b175b1fae5101e51318244d81038ac8cdd664f9d6b1c4b589d532</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>L19577560</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1785153790</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1785430800</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>5.041667</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>0xfe31a156d44f9e3b282c8377721b24b01c0625a47209ef8f421fc350af3dac0f</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0x12e3C74BC44f9C2C1f9215a84C3862510219Dd10</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>65.95</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.3713</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Europa League</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>FC Hradec Kralove</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>FC Hradec Kralove vs Tromso</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>FC Hradec Kralove</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Tromso</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0x0d9f7cd21696b245b975157ec565ba91ba0db43a168fd64ff0caebbbec205950</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>L19577176</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1785131538</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1785430800</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>177.643098</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>0x4a21e608f2a49d0d290d56e481810827c36c3a33b3cdfa52f47a9d205c9195a6</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>0x1b1185C2A2d1Ec3CA592f5c21f52dD4aD449163f</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>1.1213</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>SL Benfica FC vs FC St. Gallen</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>SL Benfica FC</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>FC St. Gallen</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>0xfc195ce6529fc46edc42b440639cd20958bc0e5f58d88c7925cdd8563a01ebd2</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>L19577588</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
         <is>
           <t>1785123830</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>1785438000</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>65.979381</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-28 06:01:17 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Europa League_UEFA/trades.xlsx
+++ b/data/sxbet/ligas/Europa League_UEFA/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,23 +531,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x9eb4b01eefa201544b1ccdb4c5c6604e0714ac629344d4d2b7b17cc1464fb5c7</t>
+          <t>0xca988989ba0a99335f19af5ab577f6640bf20ceaa254429962c758daa3ff0c0c</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFbF8d0BCccedDdAc69C0DC38823fE24842afa03C</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4.881</t>
+          <t>20.5</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5337</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,7 +559,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove vs Tromso</t>
+          <t>Ferencvaros vs FC Twente</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Tromso</t>
+          <t>FC Twente</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xc43fb7b2993be2553cb93dc8bab291577c90b4aa7ac359f3b83149bfa631bb40</t>
+          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19577176</t>
+          <t>L19578664</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785189317</t>
+          <t>1785218406</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785430800</t>
+          <t>1785436200</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>9.144731</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,28 +643,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x72247e16c302aa1a252495938a15e1d60e4b267830f4978c0b1e53c944fe7833</t>
+          <t>0x4afd29fa21cf73928533235449b4ada4ed33982b7d01229bef2dcf99368da4ca</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xFbF8d0BCccedDdAc69C0DC38823fE24842afa03C</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4.881</t>
+          <t>85.47</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5337</t>
+          <t>1.3362</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Europa League</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -667,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove vs Tromso</t>
+          <t>FC Midtjylland vs Besiktas</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove</t>
+          <t>FC Midtjylland</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Tromso</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xc43fb7b2993be2553cb93dc8bab291577c90b4aa7ac359f3b83149bfa631bb40</t>
+          <t>0x158b3cb30055ece93c8939659bae73b26e24f9856d9863a174210fcbbd5c7593</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19577176</t>
+          <t>L19577560</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785188885</t>
+          <t>1785213181</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -722,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>9.144731</t>
+          <t>254.185874</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,27 +747,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x605d65f217cfad8dba3fc5fc8ba81f33c522bb6d2702ab1896e28f2a043e7284</t>
+          <t>0x9eb4b01eefa201544b1ccdb4c5c6604e0714ac629344d4d2b7b17cc1464fb5c7</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFbF8d0BCccedDdAc69C0DC38823fE24842afa03C</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>20.5</t>
+          <t>4.881</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t>1.5337</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -767,11 +771,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>FC Twente</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -779,27 +779,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Ferencvaros vs FC Twente</t>
+          <t>FC Hradec Kralove vs Tromso</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Ferencvaros</t>
+          <t>FC Hradec Kralove</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>FC Twente</t>
+          <t>Tromso</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
+          <t>0xc43fb7b2993be2553cb93dc8bab291577c90b4aa7ac359f3b83149bfa631bb40</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19578664</t>
+          <t>L19577176</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +824,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785186773</t>
+          <t>1785189317</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785436200</t>
+          <t>1785430800</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>9.144731</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,27 +851,23 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x31389f85488fa9e54013f64ac333a2b550d2412b8db664b843e4ce83e7ac4987</t>
+          <t>0x72247e16c302aa1a252495938a15e1d60e4b267830f4978c0b1e53c944fe7833</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFbF8d0BCccedDdAc69C0DC38823fE24842afa03C</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>20.5</t>
+          <t>4.881</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t>1.5337</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -879,11 +875,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>FC Twente</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -891,27 +883,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Ferencvaros vs FC Twente</t>
+          <t>FC Hradec Kralove vs Tromso</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Ferencvaros</t>
+          <t>FC Hradec Kralove</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>FC Twente</t>
+          <t>Tromso</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
+          <t>0xc43fb7b2993be2553cb93dc8bab291577c90b4aa7ac359f3b83149bfa631bb40</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19578664</t>
+          <t>L19577176</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -936,17 +928,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785186621</t>
+          <t>1785188885</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1785436200</t>
+          <t>1785430800</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>9.144731</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,7 +955,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xfb23cf678aafc207af69fb8dfa1e83d0a06b41177f42b72e0eb9221a27e820ba</t>
+          <t>0x605d65f217cfad8dba3fc5fc8ba81f33c522bb6d2702ab1896e28f2a043e7284</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1048,7 +1040,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785186464</t>
+          <t>1785186773</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1075,7 +1067,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x3138a3ad46ea4c79099bef4064759debf254c0f7929452594d354137a19e0673</t>
+          <t>0x31389f85488fa9e54013f64ac333a2b550d2412b8db664b843e4ce83e7ac4987</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1160,7 +1152,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785186313</t>
+          <t>1785186621</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1187,7 +1179,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x2f2706b1ff85c18b198514da422a74b19942ac8b11089fe8ede6b98b57fcd6fd</t>
+          <t>0xfb23cf678aafc207af69fb8dfa1e83d0a06b41177f42b72e0eb9221a27e820ba</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1272,7 +1264,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785185868</t>
+          <t>1785186464</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1299,31 +1291,39 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x75d4a8cc9d03da588fcd6106f912b7eb69342da973970aa5144a52fd652df720</t>
+          <t>0x3138a3ad46ea4c79099bef4064759debf254c0f7929452594d354137a19e0673</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x8b3809dd81A411A1CcC110e23281D3861E41D439</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>20.5</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x31485d66881ea25fc18ee05567734ae7ae66fb87f6fcca8575303fab366000be</t>
+          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785182082</t>
+          <t>1785186313</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>101.408451</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,12 +1403,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xd994586c2c89af6ad574d50a0f8c8700e90e7f22d20bf49a633feaa989af50bf</t>
+          <t>0x2f2706b1ff85c18b198514da422a74b19942ac8b11089fe8ede6b98b57fcd6fd</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1418,22 +1418,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>98.9699</t>
+          <t>20.5</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.9187</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Europa League</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SL Benfica FC</t>
+          <t>FC Twente</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1443,27 +1443,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>SL Benfica FC vs FC St. Gallen</t>
+          <t>Ferencvaros vs FC Twente</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>SL Benfica FC</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>FC St. Gallen</t>
+          <t>FC Twente</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xf1cfaffefafaf6e63eaa25f347bda991a38fb6aa57e14fa84b386fed55a3f99b</t>
+          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19577588</t>
+          <t>L19578664</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1488,17 +1488,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785178276</t>
+          <t>1785185868</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1785438000</t>
+          <t>1785436200</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>107.72234</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1515,28 +1515,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xcfc2858bc694fbf8557c05f8f7fd20f59fd4990088d7f08f96947050324a2e61</t>
+          <t>0x75d4a8cc9d03da588fcd6106f912b7eb69342da973970aa5144a52fd652df720</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8b3809dd81A411A1CcC110e23281D3861E41D439</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1547,27 +1547,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>FC Midtjylland vs Besiktas</t>
+          <t>Ferencvaros vs FC Twente</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>FC Twente</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xda06ff264d51913dfda755a8c4a477b88663ff22d289eb6f556018e55bf68d04</t>
+          <t>0x31485d66881ea25fc18ee05567734ae7ae66fb87f6fcca8575303fab366000be</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19577560</t>
+          <t>L19578664</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1592,17 +1592,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785157337</t>
+          <t>1785182082</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1785430800</t>
+          <t>1785436200</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>101.408451</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,12 +1619,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x6d9c715f878347d23b5132d44c3d76e250960d8a888670fe9b446ebcef8c5cef</t>
+          <t>0xd994586c2c89af6ad574d50a0f8c8700e90e7f22d20bf49a633feaa989af50bf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x44cE278A4b373d2bFD26e6a2F5fA4E3550151d67</t>
+          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1634,22 +1634,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>98.9699</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.9187</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Europa League</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>SL Benfica FC</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1659,27 +1659,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>FC Midtjylland vs Besiktas</t>
+          <t>SL Benfica FC vs FC St. Gallen</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>SL Benfica FC</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>FC St. Gallen</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xd45cdb893a2b175b1fae5101e51318244d81038ac8cdd664f9d6b1c4b589d532</t>
+          <t>0xf1cfaffefafaf6e63eaa25f347bda991a38fb6aa57e14fa84b386fed55a3f99b</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19577560</t>
+          <t>L19577588</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1704,17 +1704,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785154148</t>
+          <t>1785178276</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1785430800</t>
+          <t>1785438000</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>5.041667</t>
+          <t>107.72234</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,27 +1731,23 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xc10cd30f1ad9ff73882f16291a9858024418214eb562a5dbbad80c0ecae1c52f</t>
+          <t>0xcfc2858bc694fbf8557c05f8f7fd20f59fd4990088d7f08f96947050324a2e61</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2.36789</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1759,34 +1755,30 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>FC Midtjylland vs Besiktas</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>FC Midtjylland</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t>Besiktas</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Europa League_UEFA</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>FC Midtjylland vs Besiktas</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>FC Midtjylland</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Besiktas</t>
-        </is>
-      </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xd45cdb893a2b175b1fae5101e51318244d81038ac8cdd664f9d6b1c4b589d532</t>
+          <t>0xda06ff264d51913dfda755a8c4a477b88663ff22d289eb6f556018e55bf68d04</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1816,7 +1808,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785153790</t>
+          <t>1785157337</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1826,7 +1818,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>9.866208</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1843,7 +1835,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x72c1b3c5fcfde9fcf9031572e4700cad5504a7350908921543fd656f10cf9747</t>
+          <t>0x6d9c715f878347d23b5132d44c3d76e250960d8a888670fe9b446ebcef8c5cef</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1928,7 +1920,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785153790</t>
+          <t>1785154148</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1955,12 +1947,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xfe31a156d44f9e3b282c8377721b24b01c0625a47209ef8f421fc350af3dac0f</t>
+          <t>0xc10cd30f1ad9ff73882f16291a9858024418214eb562a5dbbad80c0ecae1c52f</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x12e3C74BC44f9C2C1f9215a84C3862510219Dd10</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1970,22 +1962,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>65.95</t>
+          <t>2.36789</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.3713</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Europa League</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1995,27 +1987,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove vs Tromso</t>
+          <t>FC Midtjylland vs Besiktas</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove</t>
+          <t>FC Midtjylland</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Tromso</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x0d9f7cd21696b245b975157ec565ba91ba0db43a168fd64ff0caebbbec205950</t>
+          <t>0xd45cdb893a2b175b1fae5101e51318244d81038ac8cdd664f9d6b1c4b589d532</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19577176</t>
+          <t>L19577560</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2040,7 +2032,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785131538</t>
+          <t>1785153790</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2050,7 +2042,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>177.643098</t>
+          <t>9.866208</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2067,110 +2059,334 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>0x72c1b3c5fcfde9fcf9031572e4700cad5504a7350908921543fd656f10cf9747</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0x44cE278A4b373d2bFD26e6a2F5fA4E3550151d67</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>FC Midtjylland vs Besiktas</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>FC Midtjylland</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0xd45cdb893a2b175b1fae5101e51318244d81038ac8cdd664f9d6b1c4b589d532</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>L19577560</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1785153790</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1785430800</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>5.041667</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>0xfe31a156d44f9e3b282c8377721b24b01c0625a47209ef8f421fc350af3dac0f</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0x12e3C74BC44f9C2C1f9215a84C3862510219Dd10</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>65.95</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.3713</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Europa League</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>FC Hradec Kralove</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>FC Hradec Kralove vs Tromso</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>FC Hradec Kralove</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Tromso</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0x0d9f7cd21696b245b975157ec565ba91ba0db43a168fd64ff0caebbbec205950</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>L19577176</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1785131538</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1785430800</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>177.643098</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>0x4a21e608f2a49d0d290d56e481810827c36c3a33b3cdfa52f47a9d205c9195a6</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>0x1b1185C2A2d1Ec3CA592f5c21f52dD4aD449163f</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>1.1213</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>SL Benfica FC vs FC St. Gallen</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>SL Benfica FC</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>FC St. Gallen</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>0xfc195ce6529fc46edc42b440639cd20958bc0e5f58d88c7925cdd8563a01ebd2</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>L19577588</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
         <is>
           <t>1785123830</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>1785438000</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>65.979381</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="V18" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-28 16:01:21 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Europa League_UEFA/trades.xlsx
+++ b/data/sxbet/ligas/Europa League_UEFA/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V24"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x5b9af63c5725778fa8715fec08b7397c09f53eb358b72546a56bc49a09ede5cc</t>
+          <t>0x9e9aa5c67caefa7b6245f5765d40e430f611a0f6e43fdc57fd933b7fcbacc156</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>142.02999</t>
+          <t>5.39</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.6663</t>
+          <t>1.3425</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Europa League</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>FC Midtjylland</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -571,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>FC Midtjylland vs Besiktas</t>
+          <t>SL Benfica FC vs FC St. Gallen</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>SL Benfica FC</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>FC St. Gallen</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x4a55a2f0090a43830b1ad6efc04e3bf7a84f7e0aa2bcd1a80d7d51910165541a</t>
+          <t>0x2767b479f8b8acc38966c52e52e206d4141508d19d1c7fe6e048023fd39e34e6</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19577560</t>
+          <t>L19577588</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785232812</t>
+          <t>1785253987</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785430800</t>
+          <t>1785438000</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>213.178221</t>
+          <t>15.737226</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x6c09e3e7210d83a76913ce501fe47cdeb56af423b366465eced54e7fe5c928c8</t>
+          <t>0x5b9af63c5725778fa8715fec08b7397c09f53eb358b72546a56bc49a09ede5cc</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,12 +650,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>193.23</t>
+          <t>142.02999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.6763</t>
+          <t>1.6663</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -728,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785231712</t>
+          <t>1785232812</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>285.737523</t>
+          <t>213.178221</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,31 +747,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x48ac55426f694bdf3a16cabad44e789e8abb89d3984db5a3e886a222372d0145</t>
+          <t>0x6c09e3e7210d83a76913ce501fe47cdeb56af423b366465eced54e7fe5c928c8</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x73744622d71843A17e7CE3b9b0241AC776baC5bD</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10.9</t>
+          <t>193.23</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.6763</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Europa League</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>FC Midtjylland</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -787,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove vs Tromso</t>
+          <t>FC Midtjylland vs Besiktas</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove</t>
+          <t>FC Midtjylland</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Tromso</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xc43fb7b2993be2553cb93dc8bab291577c90b4aa7ac359f3b83149bfa631bb40</t>
+          <t>0x4a55a2f0090a43830b1ad6efc04e3bf7a84f7e0aa2bcd1a80d7d51910165541a</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19577176</t>
+          <t>L19577560</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785227020</t>
+          <t>1785231712</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>20.185185</t>
+          <t>285.737523</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,39 +859,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x885c406b02670b86a148e689b9938d8e785e5704f28af70303bb3aef7f6c7b82</t>
+          <t>0x48ac55426f694bdf3a16cabad44e789e8abb89d3984db5a3e886a222372d0145</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x73744622d71843A17e7CE3b9b0241AC776baC5bD</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>104.47</t>
+          <t>10.9</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.67</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Europa League</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>FC Midtjylland</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -899,27 +891,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>FC Midtjylland vs Besiktas</t>
+          <t>FC Hradec Kralove vs Tromso</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>FC Hradec Kralove</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>Tromso</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x4a55a2f0090a43830b1ad6efc04e3bf7a84f7e0aa2bcd1a80d7d51910165541a</t>
+          <t>0xc43fb7b2993be2553cb93dc8bab291577c90b4aa7ac359f3b83149bfa631bb40</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19577560</t>
+          <t>L19577176</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,7 +936,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785224116</t>
+          <t>1785227020</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +946,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>155.925373</t>
+          <t>20.185185</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +963,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xa9086b2a7ec89ecd1c6174888e0f5bc803e9c0bc8a10ac6884f1784dae54a2a2</t>
+          <t>0x885c406b02670b86a148e689b9938d8e785e5704f28af70303bb3aef7f6c7b82</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -986,7 +978,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>96.54</t>
+          <t>104.47</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1056,7 +1048,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785223916</t>
+          <t>1785224116</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>144.089552</t>
+          <t>155.925373</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,31 +1075,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x33629072d294c777753d4f0901c1a103d9a8351673ecfc006ec713710c194429</t>
+          <t>0xa9086b2a7ec89ecd1c6174888e0f5bc803e9c0bc8a10ac6884f1784dae54a2a2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x3Bd04051C13fcC95955fBA999a81b549DC1AaD6D</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>70.47999</t>
+          <t>96.54</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.5288</t>
+          <t>1.67</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>Europa League</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>FC Midtjylland</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -1115,27 +1115,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove vs Tromso</t>
+          <t>FC Midtjylland vs Besiktas</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove</t>
+          <t>FC Midtjylland</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Tromso</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xc43fb7b2993be2553cb93dc8bab291577c90b4aa7ac359f3b83149bfa631bb40</t>
+          <t>0x4a55a2f0090a43830b1ad6efc04e3bf7a84f7e0aa2bcd1a80d7d51910165541a</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19577176</t>
+          <t>L19577560</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785220497</t>
+          <t>1785223916</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>133.295489</t>
+          <t>144.089552</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,27 +1187,23 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xca988989ba0a99335f19af5ab577f6640bf20ceaa254429962c758daa3ff0c0c</t>
+          <t>0x33629072d294c777753d4f0901c1a103d9a8351673ecfc006ec713710c194429</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x3Bd04051C13fcC95955fBA999a81b549DC1AaD6D</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>20.5</t>
+          <t>70.47999</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t>1.5288</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1215,11 +1211,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>FC Twente</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -1227,27 +1219,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Ferencvaros vs FC Twente</t>
+          <t>FC Hradec Kralove vs Tromso</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Ferencvaros</t>
+          <t>FC Hradec Kralove</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>FC Twente</t>
+          <t>Tromso</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
+          <t>0xc43fb7b2993be2553cb93dc8bab291577c90b4aa7ac359f3b83149bfa631bb40</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19578664</t>
+          <t>L19577176</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1272,17 +1264,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785218406</t>
+          <t>1785220497</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1785436200</t>
+          <t>1785430800</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>133.295489</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,7 +1291,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x4afd29fa21cf73928533235449b4ada4ed33982b7d01229bef2dcf99368da4ca</t>
+          <t>0xca988989ba0a99335f19af5ab577f6640bf20ceaa254429962c758daa3ff0c0c</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1307,23 +1299,31 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>85.47</t>
+          <t>20.5</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.3362</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Europa League</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -1331,27 +1331,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>FC Midtjylland vs Besiktas</t>
+          <t>Ferencvaros vs FC Twente</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>FC Twente</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x158b3cb30055ece93c8939659bae73b26e24f9856d9863a174210fcbbd5c7593</t>
+          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19577560</t>
+          <t>L19578664</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1376,17 +1376,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785213181</t>
+          <t>1785218406</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1785430800</t>
+          <t>1785436200</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>254.185874</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,28 +1403,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x9eb4b01eefa201544b1ccdb4c5c6604e0714ac629344d4d2b7b17cc1464fb5c7</t>
+          <t>0x4afd29fa21cf73928533235449b4ada4ed33982b7d01229bef2dcf99368da4ca</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xFbF8d0BCccedDdAc69C0DC38823fE24842afa03C</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4.881</t>
+          <t>85.47</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.5337</t>
+          <t>1.3362</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Europa League</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1435,27 +1435,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove vs Tromso</t>
+          <t>FC Midtjylland vs Besiktas</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove</t>
+          <t>FC Midtjylland</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Tromso</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xc43fb7b2993be2553cb93dc8bab291577c90b4aa7ac359f3b83149bfa631bb40</t>
+          <t>0x158b3cb30055ece93c8939659bae73b26e24f9856d9863a174210fcbbd5c7593</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19577176</t>
+          <t>L19577560</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785189317</t>
+          <t>1785213181</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>9.144731</t>
+          <t>254.185874</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,7 +1507,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x72247e16c302aa1a252495938a15e1d60e4b267830f4978c0b1e53c944fe7833</t>
+          <t>0x9eb4b01eefa201544b1ccdb4c5c6604e0714ac629344d4d2b7b17cc1464fb5c7</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785188885</t>
+          <t>1785189317</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1611,27 +1611,23 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x605d65f217cfad8dba3fc5fc8ba81f33c522bb6d2702ab1896e28f2a043e7284</t>
+          <t>0x72247e16c302aa1a252495938a15e1d60e4b267830f4978c0b1e53c944fe7833</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFbF8d0BCccedDdAc69C0DC38823fE24842afa03C</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>20.5</t>
+          <t>4.881</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t>1.5337</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1639,11 +1635,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>FC Twente</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -1651,27 +1643,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Ferencvaros vs FC Twente</t>
+          <t>FC Hradec Kralove vs Tromso</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Ferencvaros</t>
+          <t>FC Hradec Kralove</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>FC Twente</t>
+          <t>Tromso</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
+          <t>0xc43fb7b2993be2553cb93dc8bab291577c90b4aa7ac359f3b83149bfa631bb40</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19578664</t>
+          <t>L19577176</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1696,17 +1688,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785186773</t>
+          <t>1785188885</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1785436200</t>
+          <t>1785430800</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>9.144731</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1723,7 +1715,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x31389f85488fa9e54013f64ac333a2b550d2412b8db664b843e4ce83e7ac4987</t>
+          <t>0x605d65f217cfad8dba3fc5fc8ba81f33c522bb6d2702ab1896e28f2a043e7284</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1808,7 +1800,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785186621</t>
+          <t>1785186773</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1835,7 +1827,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xfb23cf678aafc207af69fb8dfa1e83d0a06b41177f42b72e0eb9221a27e820ba</t>
+          <t>0x31389f85488fa9e54013f64ac333a2b550d2412b8db664b843e4ce83e7ac4987</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1920,7 +1912,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785186464</t>
+          <t>1785186621</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1947,7 +1939,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x3138a3ad46ea4c79099bef4064759debf254c0f7929452594d354137a19e0673</t>
+          <t>0xfb23cf678aafc207af69fb8dfa1e83d0a06b41177f42b72e0eb9221a27e820ba</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2032,7 +2024,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785186313</t>
+          <t>1785186464</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2059,7 +2051,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x2f2706b1ff85c18b198514da422a74b19942ac8b11089fe8ede6b98b57fcd6fd</t>
+          <t>0x3138a3ad46ea4c79099bef4064759debf254c0f7929452594d354137a19e0673</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2144,7 +2136,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785185868</t>
+          <t>1785186313</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2171,31 +2163,39 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x75d4a8cc9d03da588fcd6106f912b7eb69342da973970aa5144a52fd652df720</t>
+          <t>0x2f2706b1ff85c18b198514da422a74b19942ac8b11089fe8ede6b98b57fcd6fd</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x8b3809dd81A411A1CcC110e23281D3861E41D439</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>20.5</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x31485d66881ea25fc18ee05567734ae7ae66fb87f6fcca8575303fab366000be</t>
+          <t>0xe84ac6325784d17111f3c60f2ba80ccbf3ba57796f09390d50991fbef4aa01e7</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785182082</t>
+          <t>1785185868</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>101.408451</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2275,39 +2275,31 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xd994586c2c89af6ad574d50a0f8c8700e90e7f22d20bf49a633feaa989af50bf</t>
+          <t>0x75d4a8cc9d03da588fcd6106f912b7eb69342da973970aa5144a52fd652df720</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8b3809dd81A411A1CcC110e23281D3861E41D439</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>98.9699</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.9187</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Europa League</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>SL Benfica FC</t>
-        </is>
-      </c>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -2315,27 +2307,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>SL Benfica FC vs FC St. Gallen</t>
+          <t>Ferencvaros vs FC Twente</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>SL Benfica FC</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>FC St. Gallen</t>
+          <t>FC Twente</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xf1cfaffefafaf6e63eaa25f347bda991a38fb6aa57e14fa84b386fed55a3f99b</t>
+          <t>0x31485d66881ea25fc18ee05567734ae7ae66fb87f6fcca8575303fab366000be</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19577588</t>
+          <t>L19578664</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2360,17 +2352,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785178276</t>
+          <t>1785182082</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1785438000</t>
+          <t>1785436200</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>107.72234</t>
+          <t>101.408451</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2387,31 +2379,39 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xcfc2858bc694fbf8557c05f8f7fd20f59fd4990088d7f08f96947050324a2e61</t>
+          <t>0xd994586c2c89af6ad574d50a0f8c8700e90e7f22d20bf49a633feaa989af50bf</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>98.9699</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.9187</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>Europa League</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>SL Benfica FC</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
@@ -2419,27 +2419,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>FC Midtjylland vs Besiktas</t>
+          <t>SL Benfica FC vs FC St. Gallen</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>SL Benfica FC</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>FC St. Gallen</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xda06ff264d51913dfda755a8c4a477b88663ff22d289eb6f556018e55bf68d04</t>
+          <t>0xf1cfaffefafaf6e63eaa25f347bda991a38fb6aa57e14fa84b386fed55a3f99b</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19577560</t>
+          <t>L19577588</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2464,17 +2464,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785157337</t>
+          <t>1785178276</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1785430800</t>
+          <t>1785438000</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>107.72234</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2491,27 +2491,23 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x6d9c715f878347d23b5132d44c3d76e250960d8a888670fe9b446ebcef8c5cef</t>
+          <t>0xcfc2858bc694fbf8557c05f8f7fd20f59fd4990088d7f08f96947050324a2e61</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x44cE278A4b373d2bFD26e6a2F5fA4E3550151d67</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2519,34 +2515,30 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>FC Midtjylland vs Besiktas</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>FC Midtjylland</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
         <is>
           <t>Besiktas</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Europa League_UEFA</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>FC Midtjylland vs Besiktas</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>FC Midtjylland</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Besiktas</t>
-        </is>
-      </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xd45cdb893a2b175b1fae5101e51318244d81038ac8cdd664f9d6b1c4b589d532</t>
+          <t>0xda06ff264d51913dfda755a8c4a477b88663ff22d289eb6f556018e55bf68d04</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2576,7 +2568,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785154148</t>
+          <t>1785157337</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2586,7 +2578,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>5.041667</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2603,12 +2595,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xc10cd30f1ad9ff73882f16291a9858024418214eb562a5dbbad80c0ecae1c52f</t>
+          <t>0x6d9c715f878347d23b5132d44c3d76e250960d8a888670fe9b446ebcef8c5cef</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0x44cE278A4b373d2bFD26e6a2F5fA4E3550151d67</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2618,7 +2610,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2.36789</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2688,7 +2680,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785153790</t>
+          <t>1785154148</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2698,7 +2690,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>9.866208</t>
+          <t>5.041667</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2715,12 +2707,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x72c1b3c5fcfde9fcf9031572e4700cad5504a7350908921543fd656f10cf9747</t>
+          <t>0xc10cd30f1ad9ff73882f16291a9858024418214eb562a5dbbad80c0ecae1c52f</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x44cE278A4b373d2bFD26e6a2F5fA4E3550151d67</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2730,7 +2722,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>2.36789</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2810,7 +2802,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>5.041667</t>
+          <t>9.866208</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2827,12 +2819,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xfe31a156d44f9e3b282c8377721b24b01c0625a47209ef8f421fc350af3dac0f</t>
+          <t>0x72c1b3c5fcfde9fcf9031572e4700cad5504a7350908921543fd656f10cf9747</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x12e3C74BC44f9C2C1f9215a84C3862510219Dd10</t>
+          <t>0x44cE278A4b373d2bFD26e6a2F5fA4E3550151d67</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2842,22 +2834,22 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>65.95</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.3713</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Europa League</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2867,27 +2859,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove vs Tromso</t>
+          <t>FC Midtjylland vs Besiktas</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>FC Hradec Kralove</t>
+          <t>FC Midtjylland</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Tromso</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x0d9f7cd21696b245b975157ec565ba91ba0db43a168fd64ff0caebbbec205950</t>
+          <t>0xd45cdb893a2b175b1fae5101e51318244d81038ac8cdd664f9d6b1c4b589d532</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19577176</t>
+          <t>L19577560</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2912,7 +2904,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785131538</t>
+          <t>1785153790</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2922,7 +2914,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>177.643098</t>
+          <t>5.041667</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2939,110 +2931,222 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>0xfe31a156d44f9e3b282c8377721b24b01c0625a47209ef8f421fc350af3dac0f</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0x12e3C74BC44f9C2C1f9215a84C3862510219Dd10</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>65.95</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.3713</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Europa League</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>FC Hradec Kralove</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Europa League_UEFA</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>FC Hradec Kralove vs Tromso</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>FC Hradec Kralove</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Tromso</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0x0d9f7cd21696b245b975157ec565ba91ba0db43a168fd64ff0caebbbec205950</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>L19577176</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>1785131538</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>1785430800</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>177.643098</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>0x4a21e608f2a49d0d290d56e481810827c36c3a33b3cdfa52f47a9d205c9195a6</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>0x1b1185C2A2d1Ec3CA592f5c21f52dD4aD449163f</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>1.1213</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>Europa League_UEFA</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>SL Benfica FC vs FC St. Gallen</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>SL Benfica FC</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>FC St. Gallen</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>0xfc195ce6529fc46edc42b440639cd20958bc0e5f58d88c7925cdd8563a01ebd2</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>L19577588</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
         <is>
           <t>1785123830</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
+      <c r="S25" t="inlineStr">
         <is>
           <t>1785438000</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr">
+      <c r="T25" t="inlineStr">
         <is>
           <t>65.979381</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="U25" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr">
+      <c r="V25" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>